<commit_message>
Remove dist and update public workbook
</commit_message>
<xml_diff>
--- a/public/产品库存及周转统计.xlsx
+++ b/public/产品库存及周转统计.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15240"/>
+    <workbookView windowHeight="23040"/>
   </bookViews>
   <sheets>
     <sheet name="产品库存" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">产品库存!$A$1:$AH$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">产品库存!$A$1:$AH$62</definedName>
   </definedNames>
   <calcPr calcId="144525" concurrentCalc="0"/>
 </workbook>
@@ -5941,11 +5941,11 @@
         <v>0</v>
       </c>
       <c r="T44" s="7">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="U44" s="38">
         <f t="shared" si="14"/>
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="V44" s="37"/>
       <c r="W44" s="37"/>
@@ -5962,7 +5962,7 @@
         <v>205</v>
       </c>
       <c r="AF44" s="7">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AG44" s="7">
         <v>37</v>
@@ -7555,7 +7555,7 @@
     <row r="70" ht="25" customHeight="1"/>
     <row r="71" ht="25" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:AH60">
+  <autoFilter ref="A1:AH62">
     <extLst/>
   </autoFilter>
   <conditionalFormatting sqref="J45">

</xml_diff>